<commit_message>
Add response review flags to question inventory
</commit_message>
<xml_diff>
--- a/MARP_question_inventory.xlsx
+++ b/MARP_question_inventory.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="Rfc3b8111227444ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R6136e99d230e4aff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,17 +105,28 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="1">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF0C2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MARPQuestions" displayName="MARPQuestions" ref="A5:E38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MARPQuestions" displayName="MARPQuestions" ref="A5:G38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="Field ID"/>
     <x:tableColumn id="2" name="Section"/>
     <x:tableColumn id="3" name="Question or field wording"/>
     <x:tableColumn id="4" name="Response type"/>
     <x:tableColumn id="5" name="Condition or format"/>
+    <x:tableColumn id="6" name="Review required"/>
+    <x:tableColumn id="7" name="Review reason"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -321,6 +332,8 @@
     <x:col min="3" max="3" width="95" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -329,6 +342,8 @@
       <x:c r="C1" s="1"/>
       <x:c r="D1" s="1"/>
       <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
@@ -338,6 +353,8 @@
       <x:c r="C2" s="1"/>
       <x:c r="D2" s="1"/>
       <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
@@ -347,6 +364,8 @@
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
       <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
@@ -356,6 +375,8 @@
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1"/>
       <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="7" t="str">
@@ -373,6 +394,12 @@
       <x:c r="E5" s="7" t="str">
         <x:v>Condition or format</x:v>
       </x:c>
+      <x:c r="F5" s="7" t="str">
+        <x:v>Review required</x:v>
+      </x:c>
+      <x:c r="G5" s="7" t="str">
+        <x:v>Review reason</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="10" t="str">
@@ -388,6 +415,10 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str"/>
+      <x:c r="F6" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="str"/>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="11" t="str">
@@ -405,6 +436,10 @@
       <x:c r="E7" s="11" t="str">
         <x:v>Project contact</x:v>
       </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="str"/>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="10" t="str">
@@ -422,6 +457,10 @@
       <x:c r="E8" s="10" t="str">
         <x:v>Project contact</x:v>
       </x:c>
+      <x:c r="F8" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="str"/>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="11" t="str">
@@ -439,6 +478,10 @@
       <x:c r="E9" s="11" t="str">
         <x:v>Project contact</x:v>
       </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="str"/>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
       <x:c r="A10" s="10" t="str">
@@ -456,6 +499,10 @@
       <x:c r="E10" s="10" t="str">
         <x:v>Project contact</x:v>
       </x:c>
+      <x:c r="F10" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="str"/>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="11" t="str">
@@ -473,6 +520,10 @@
       <x:c r="E11" s="11" t="str">
         <x:v>Optional; project contact</x:v>
       </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="str"/>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
       <x:c r="A12" s="10" t="str">
@@ -490,6 +541,10 @@
       <x:c r="E12" s="10" t="str">
         <x:v>Project contact</x:v>
       </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str"/>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
       <x:c r="A13" s="11" t="str">
@@ -505,6 +560,10 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str"/>
+      <x:c r="F13" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G13" s="11" t="str"/>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="10" t="str">
@@ -522,6 +581,10 @@
       <x:c r="E14" s="10" t="str">
         <x:v>YYYY-MM-DD</x:v>
       </x:c>
+      <x:c r="F14" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="str"/>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="11" t="str">
@@ -539,6 +602,10 @@
       <x:c r="E15" s="11" t="str">
         <x:v>YYYY-MM-DD</x:v>
       </x:c>
+      <x:c r="F15" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="str"/>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="10" t="str">
@@ -554,6 +621,10 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str"/>
+      <x:c r="F16" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str"/>
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
       <x:c r="A17" s="11" t="str">
@@ -571,6 +642,10 @@
       <x:c r="E17" s="11" t="str">
         <x:v>If applicable</x:v>
       </x:c>
+      <x:c r="F17" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="str"/>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="10" t="str">
@@ -586,6 +661,10 @@
         <x:v>Written response</x:v>
       </x:c>
       <x:c r="E18" s="10" t="str"/>
+      <x:c r="F18" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G18" s="10" t="str"/>
     </x:row>
     <x:row r="19" ht="44" customHeight="1">
       <x:c r="A19" s="11" t="str">
@@ -601,6 +680,10 @@
         <x:v>Yes / No</x:v>
       </x:c>
       <x:c r="E19" s="11" t="str"/>
+      <x:c r="F19" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G19" s="11" t="str"/>
     </x:row>
     <x:row r="20" ht="44" customHeight="1">
       <x:c r="A20" s="10" t="str">
@@ -618,6 +701,10 @@
       <x:c r="E20" s="10" t="str">
         <x:v>If C02 = Yes</x:v>
       </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str"/>
     </x:row>
     <x:row r="21" ht="92" customHeight="1">
       <x:c r="A21" s="11" t="str">
@@ -633,6 +720,10 @@
         <x:v>Written response</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str"/>
+      <x:c r="F21" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G21" s="11" t="str"/>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
       <x:c r="A22" s="10" t="str">
@@ -648,6 +739,10 @@
         <x:v>Yes / No</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str"/>
+      <x:c r="F22" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="str"/>
     </x:row>
     <x:row r="23" ht="44" customHeight="1">
       <x:c r="A23" s="11" t="str">
@@ -665,6 +760,10 @@
       <x:c r="E23" s="11" t="str">
         <x:v>If D02 = Yes</x:v>
       </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G23" s="11" t="str"/>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
       <x:c r="A24" s="10" t="str">
@@ -682,6 +781,10 @@
       <x:c r="E24" s="10" t="str">
         <x:v>If event involved a single community</x:v>
       </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="str"/>
     </x:row>
     <x:row r="25" ht="44" customHeight="1">
       <x:c r="A25" s="11" t="str">
@@ -699,6 +802,10 @@
       <x:c r="E25" s="11" t="str">
         <x:v>Attendance requires live presence in person and/or virtually.</x:v>
       </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str"/>
     </x:row>
     <x:row r="26" ht="44" customHeight="1">
       <x:c r="A26" s="10" t="str">
@@ -716,6 +823,10 @@
       <x:c r="E26" s="10" t="str">
         <x:v>Recurring events only; preserve whether years or occurrences were reported.</x:v>
       </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str"/>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
       <x:c r="A27" s="11" t="str">
@@ -733,6 +844,10 @@
       <x:c r="E27" s="11" t="str">
         <x:v>Recurring events only; skip if non-recurring or first occurrence.</x:v>
       </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="str"/>
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
       <x:c r="A28" s="10" t="str">
@@ -748,6 +863,10 @@
         <x:v>Written response</x:v>
       </x:c>
       <x:c r="E28" s="10" t="str"/>
+      <x:c r="F28" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="str"/>
     </x:row>
     <x:row r="29" ht="44" customHeight="1">
       <x:c r="A29" s="11" t="str">
@@ -765,6 +884,10 @@
       <x:c r="E29" s="11" t="str">
         <x:v>If applicable</x:v>
       </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G29" s="11" t="str"/>
     </x:row>
     <x:row r="30" ht="44" customHeight="1">
       <x:c r="A30" s="10" t="str">
@@ -782,6 +905,10 @@
       <x:c r="E30" s="10" t="str">
         <x:v>If any</x:v>
       </x:c>
+      <x:c r="F30" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G30" s="10" t="str"/>
     </x:row>
     <x:row r="31" ht="44" customHeight="1">
       <x:c r="A31" s="11" t="str">
@@ -797,6 +924,10 @@
         <x:v>Written response</x:v>
       </x:c>
       <x:c r="E31" s="11" t="str"/>
+      <x:c r="F31" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G31" s="11" t="str"/>
     </x:row>
     <x:row r="32" ht="76" customHeight="1">
       <x:c r="A32" s="10" t="str">
@@ -812,6 +943,10 @@
         <x:v>Yes / No</x:v>
       </x:c>
       <x:c r="E32" s="10" t="str"/>
+      <x:c r="F32" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G32" s="10" t="str"/>
     </x:row>
     <x:row r="33" ht="76" customHeight="1">
       <x:c r="A33" s="11" t="str">
@@ -829,6 +964,10 @@
       <x:c r="E33" s="11" t="str">
         <x:v>If G01 = Yes</x:v>
       </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="str"/>
     </x:row>
     <x:row r="34" ht="76" customHeight="1">
       <x:c r="A34" s="10" t="str">
@@ -846,6 +985,10 @@
       <x:c r="E34" s="10" t="str">
         <x:v>If G01 = No</x:v>
       </x:c>
+      <x:c r="F34" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G34" s="10" t="str"/>
     </x:row>
     <x:row r="35" ht="92" customHeight="1">
       <x:c r="A35" s="11" t="str">
@@ -863,6 +1006,10 @@
       <x:c r="E35" s="11" t="str">
         <x:v>If the audience included both English-speaking and French-speaking people.</x:v>
       </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="str"/>
     </x:row>
     <x:row r="36" ht="44" customHeight="1">
       <x:c r="A36" s="10" t="str">
@@ -880,6 +1027,10 @@
       <x:c r="E36" s="10" t="str">
         <x:v>Required; authorized signatory as described in the form.</x:v>
       </x:c>
+      <x:c r="F36" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G36" s="10" t="str"/>
     </x:row>
     <x:row r="37" ht="36" customHeight="1">
       <x:c r="A37" s="11" t="str">
@@ -897,6 +1048,10 @@
       <x:c r="E37" s="11" t="str">
         <x:v>Name and signature (required)</x:v>
       </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G37" s="11" t="str"/>
     </x:row>
     <x:row r="38" ht="36" customHeight="1">
       <x:c r="A38" s="10" t="str">
@@ -914,11 +1069,23 @@
       <x:c r="E38" s="10" t="str">
         <x:v>YYYY-MM-DD; sign-off date</x:v>
       </x:c>
+      <x:c r="F38" s="10" t="str">
+        <x:v>Not assessed</x:v>
+      </x:c>
+      <x:c r="G38" s="10" t="str"/>
     </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="F6:F38">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Yes"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F6:F38">
+      <x:formula1>"Not assessed,Yes,No"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf000a7c4a1d7455e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R935c68e0a956425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>